<commit_message>
Day 02 & 03 updates
</commit_message>
<xml_diff>
--- a/DSA_Level1_Tracker.xlsx
+++ b/DSA_Level1_Tracker.xlsx
@@ -634,18 +634,26 @@
           <t>6</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G3" s="2" t="n"/>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Number Theory I. Problems + operator drills set in Day02/. Difficulty nudged up (Day1 71/100 ADVANCE). Required: prime O(sqrt n), digit-loop for Armstrong/palindrome. Carryover: fix Day1 Q4 (O(n) one-pass) &amp; Q10 (real power-of-two).</t>
+          <t>Day2 ~91/100 LEVEL UP. 10/10 core PASS incl edges; stretch Q11/Q12 skipped. Strong: O(sqrt n) prime, math digit loops, bit-trick power-of-two (fixes Day1 Q10). Nits: redundant ==True / ternary-of-bool, float sqrt risk in is_prime. Difficulty bumped aggressively for Day3.</t>
         </is>
       </c>
     </row>
@@ -663,24 +671,28 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Number Theory II (GCD/LCM/Fibonacci)</t>
+          <t>Arrays + Hashing/Dict (+ NT II warm-up: GCD/LCM/Fib)</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>12</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="3" t="inlineStr"/>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Pulled forward arrays + dictionaries per request (level-up). 12 Qs: GCD/LCM/Fib, one-pass max/min (Day1 Q4 fix), second largest, move zeros, missing number, rotate; dict freq, two-sum, first non-repeating, anagram, majority. Required O(n) / O(1) space where stated.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">

</xml_diff>